<commit_message>
Atualizar planilha de Declaração de Imposto de Renda com novas informações
</commit_message>
<xml_diff>
--- a/Excel com IA/Declaração de Imposto de Renda com Excel/Declaração de Imposto de Renda.xlsx
+++ b/Excel com IA/Declaração de Imposto de Renda com Excel/Declaração de Imposto de Renda.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c2c93962861e008/Excel com IA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="320" documentId="14_{7C1CAA58-67CC-4BC7-A5D0-A01E8BB884EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C67F7A31-565B-43C2-949E-B4B11F102CF2}"/>
+  <xr:revisionPtr revIDLastSave="333" documentId="14_{7C1CAA58-67CC-4BC7-A5D0-A01E8BB884EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C418AA-E49C-4A62-A880-AF99D19CE975}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="20" firstSheet="2" activeTab="2" xr2:uid="{FE2F66FB-9D39-498F-B57F-02ED38101F5F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="20" xr2:uid="{FE2F66FB-9D39-498F-B57F-02ED38101F5F}"/>
   </bookViews>
   <sheets>
     <sheet name="TITULAR" sheetId="1" r:id="rId1"/>
@@ -89,18 +89,9 @@
     <t>Preencha os dados da sua pessoa física abaixo</t>
   </si>
   <si>
-    <t>ELEILTON SANTOS GATINHO</t>
-  </si>
-  <si>
-    <t>ilton.sa@outlook.com</t>
-  </si>
-  <si>
     <t>NÃO</t>
   </si>
   <si>
-    <t>Stephanie</t>
-  </si>
-  <si>
     <t>Rua Dez, Quadra 13, Nº 10</t>
   </si>
   <si>
@@ -315,6 +306,15 @@
   </si>
   <si>
     <t>HOLERITE</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>joao@gmail.com</t>
+  </si>
+  <si>
+    <t>JOAO  DO NASCIMENTO</t>
   </si>
 </sst>
 </file>
@@ -3310,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -3318,7 +3318,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="12">
-        <v>60580327337</v>
+        <v>12345678911</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -3326,7 +3326,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="13">
-        <v>33947</v>
+        <v>33946</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3342,7 +3342,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -3350,7 +3350,7 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3358,7 +3358,7 @@
         <v>12</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -3374,7 +3374,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="15">
-        <v>48988744350</v>
+        <v>21984456523</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
@@ -3382,7 +3382,7 @@
         <v>7</v>
       </c>
       <c r="D15" s="15">
-        <v>48988744350</v>
+        <v>21984456523</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -3390,7 +3390,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>17</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
@@ -3398,7 +3398,7 @@
         <v>9</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="3:4" x14ac:dyDescent="0.25">
@@ -3406,7 +3406,7 @@
         <v>10</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="3:4" x14ac:dyDescent="0.25">
@@ -3414,7 +3414,7 @@
         <v>11</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -3429,7 +3429,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D16" r:id="rId1" xr:uid="{64F61639-6C60-4CC6-91B7-635371107D20}"/>
+    <hyperlink ref="D16" r:id="rId1" display="ilton.sa@outlook.com" xr:uid="{64F61639-6C60-4CC6-91B7-635371107D20}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId2"/>
@@ -3448,21 +3448,21 @@
   <sheetData>
     <row r="3" spans="3:5" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="5" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
     </row>
     <row r="4" spans="3:5" ht="21.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C4" s="24" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4" s="24"/>
       <c r="E4" s="24"/>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C6" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.25">
@@ -3474,20 +3474,20 @@
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C9" s="9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C11" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" s="17">
         <v>500000</v>
@@ -3495,28 +3495,28 @@
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C12" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C14" s="9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C15" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C16" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D16" s="17">
         <v>1000000</v>
@@ -3524,28 +3524,28 @@
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C17" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C19" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C20" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C21" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D21" s="17">
         <v>800000</v>
@@ -3553,10 +3553,10 @@
     </row>
     <row r="22" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C22" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -3594,34 +3594,34 @@
   <sheetData>
     <row r="3" spans="3:5" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
     </row>
     <row r="4" spans="3:5" ht="21.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C4" s="24" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4" s="24"/>
       <c r="E4" s="24"/>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C7" s="27" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="27"/>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C8" s="22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.25">
@@ -3629,7 +3629,7 @@
         <v>46046</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E9" s="20">
         <v>3000</v>
@@ -3809,257 +3809,257 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>